<commit_message>
Add Market Sizing & EU Revenue tab with capture analysis
New sheet 'Market Sizing & EU Revenue' added to the xlsx workbook,
with corresponding CSV. Covers 16 sub-segments across Semiconductors,
Cloud, AI Datacenters, LLMs, and Quantum with:
- Global market size (2025 actual, 2026E forecast)
- EU market size and share of global
- EU revenue captured by EU-HQ companies vs non-EU companies
- Color-coded capture columns (green = EU, red = non-EU)
- Key takeaways summary ranking segments by EU capture strength

Data sourced from SIA/WSTS, Synergy Research, Deloitte, ASML/Infineon/
NXP/STMicro annual reports, QED-C, Silicon Analysts, and others.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EU_Chips_Act_2.0_Dependency_Analysis.xlsx
+++ b/EU_Chips_Act_2.0_Dependency_Analysis.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet name="Dependency Analysis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Market Sizing &amp; EU Revenue" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dependency Analysis'!$A$1:$N$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Market Sizing &amp; EU Revenue'!$A$1:$O$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +60,32 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -129,6 +158,30 @@
         <bgColor rgb="0000B050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6600"/>
+        <bgColor rgb="00FF6600"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -156,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -214,6 +267,94 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3272,4 +3413,1239 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="55" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AREA</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SUB-SEGMENT</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>GLOBAL MARKET SIZE 2025
+(USD bn)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>GLOBAL MARKET SIZE 2026E
+(USD bn)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>EU MARKET SIZE 2025
+(USD bn)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>EU MARKET SIZE 2026E
+(USD bn)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>EU AS % OF
+GLOBAL (2025)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>EU AS % OF
+GLOBAL (2026E)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>EU REVENUE CAPTURED BY
+EU-HQ COMPANIES (USD bn, 2025)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>EU REVENUE CAPTURED BY
+NON-EU COMPANIES (USD bn, 2025)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>% CAPTURED BY
+EU COMPANIES</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>% CAPTURED BY
+NON-EU COMPANIES</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>KEY EU COMPANIES
+(Revenue, 2025)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>KEY NON-EU COMPANIES
+(Share of EU Market)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>SOURCE / NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="70" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>SEMICONDUCTORS</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Total Semiconductor Market</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="n">
+        <v>791.7</v>
+      </c>
+      <c r="D2" s="20" t="n">
+        <v>975</v>
+      </c>
+      <c r="E2" s="20" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="F2" s="20" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="G2" s="21" t="n">
+        <v>0.06883920677024125</v>
+      </c>
+      <c r="H2" s="21" t="n">
+        <v>0.06194871794871794</v>
+      </c>
+      <c r="I2" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="J2" s="23" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="K2" s="24" t="n">
+        <v>0.2935779816513762</v>
+      </c>
+      <c r="L2" s="25" t="n">
+        <v>0.7064220183486238</v>
+      </c>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>Infineon (€14.7bn global), NXP ($12.3bn global), STMicro ($11.8bn global); combined EU-market share ~30%</t>
+        </is>
+      </c>
+      <c r="N2" s="15" t="inlineStr">
+        <is>
+          <t>Intel, TSMC, Samsung, Qualcomm, Broadcom, Texas Instruments supply ~70% of EU chip consumption</t>
+        </is>
+      </c>
+      <c r="O2" s="26" t="inlineStr">
+        <is>
+          <t>SIA/WSTS 2025 actuals; WSTS Autumn 2026 forecast ($975bn); ESIA Europe data ($54.5bn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="70" customHeight="1">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>SEMICONDUCTORS</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>AI Chips (Logic + AI Memory)</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="D3" s="20" t="n">
+        <v>280</v>
+      </c>
+      <c r="E3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" s="21" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="H3" s="21" t="n">
+        <v>0.02857142857142857</v>
+      </c>
+      <c r="I3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>No scaled EU AI chip company; Axelera AI, SiPearl are pre-scale (&lt;$50M combined)</t>
+        </is>
+      </c>
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>NVIDIA ($130bn+ DC rev), AMD ($10bn+), Google/AWS/Meta custom silicon ($15bn+); 100% of EU AI chip supply</t>
+        </is>
+      </c>
+      <c r="O3" s="26" t="inlineStr">
+        <is>
+          <t>Silicon Analysts; Deloitte 2026 Outlook; AI chips ~50% of total semi revenue by value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>SEMICONDUCTORS</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Semiconductor Equipment</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="n">
+        <v>110</v>
+      </c>
+      <c r="D4" s="20" t="n">
+        <v>125</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>38</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>43</v>
+      </c>
+      <c r="G4" s="21" t="n">
+        <v>36</v>
+      </c>
+      <c r="H4" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" s="24" t="inlineStr">
+        <is>
+          <t>ASML (€32.7bn / ~$35.5bn global rev); Zeiss, BESI, ASM Intl (~$2.5bn combined EU rev)</t>
+        </is>
+      </c>
+      <c r="L4" s="25" t="inlineStr">
+        <is>
+          <t>Applied Materials, Lam Research, Tokyo Electron, KLA, Screen (~$2bn EU-origin rev)</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>ASML Annual Report 2025; EU dominates via ASML EUV monopoly; equipment is EU strength area</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="inlineStr"/>
+      <c r="O4" s="26" t="inlineStr"/>
+    </row>
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>SEMICONDUCTORS</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Power / Automotive / Industrial Chips</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>95</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <v>102</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="I5" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K5" s="24" t="inlineStr">
+        <is>
+          <t>Infineon (~$10bn EU auto/industrial), NXP (~$5bn EU), STMicro (~$4bn EU); ~60% of EU segment</t>
+        </is>
+      </c>
+      <c r="L5" s="25" t="inlineStr">
+        <is>
+          <t>Texas Instruments, ON Semi, Renesas, Microchip; ~40% of EU power/auto segment</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>Company annual reports; EU has strong position in automotive/power semis</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr"/>
+      <c r="O5" s="26" t="inlineStr"/>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>SEMICONDUCTORS</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>High Bandwidth Memory (HBM)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>0.05357142857142857</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>0.05555555555555555</v>
+      </c>
+      <c r="I6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>No EU HBM producer</t>
+        </is>
+      </c>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>SK Hynix (~50% global), Samsung (~40%), Micron (~10%); 100% of EU HBM is imported</t>
+        </is>
+      </c>
+      <c r="O6" s="26" t="inlineStr">
+        <is>
+          <t>Deloitte; industry estimates; HBM critical for AI training/inference</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>CLOUD</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cloud Infrastructure Services (IaaS/PaaS/Hosted Private Cloud)</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>350</v>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>435</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>87</v>
+      </c>
+      <c r="F7" s="29" t="n">
+        <v>108</v>
+      </c>
+      <c r="G7" s="30" t="n">
+        <v>0.2485714285714286</v>
+      </c>
+      <c r="H7" s="30" t="n">
+        <v>0.2482758620689655</v>
+      </c>
+      <c r="I7" s="22" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="J7" s="23" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="K7" s="24" t="n">
+        <v>0.1505747126436782</v>
+      </c>
+      <c r="L7" s="25" t="n">
+        <v>0.8494252873563219</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>OVHcloud (~$1bn), SAP (~$1.7bn cloud infra), Deutsche Telekom/T-Systems (~$1.7bn), Scaleway, STACKIT, others (~$8.7bn)</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>AWS (~30%), Azure (~25%), Google Cloud (~15%); combined ~70% of EU cloud infra = ~$61bn</t>
+        </is>
+      </c>
+      <c r="O7" s="31" t="inlineStr">
+        <is>
+          <t>Synergy Research Group 2025; EU market ~€61bn ($70bn) in 2024, growing 24% YoY; EU providers at 15% share</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CLOUD</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SaaS (Software as a Service)</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>430</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>500</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>86</v>
+      </c>
+      <c r="F8" s="29" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H8" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="K8" s="24" t="n">
+        <v>0.09999999999999999</v>
+      </c>
+      <c r="L8" s="25" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>SAP ($8bn+ EU SaaS), Dassault Systemes, Sage, TeamViewer, others; ~10% of EU SaaS spend</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft 365, Salesforce, Google Workspace, ServiceNow, Oracle; ~90% of EU SaaS spend</t>
+        </is>
+      </c>
+      <c r="O8" s="31" t="inlineStr">
+        <is>
+          <t>Grand View Research; Fortune BI; SAP is largest EU SaaS provider; US dominance even more acute than IaaS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CLOUD</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Sovereign Cloud Services</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G9" s="30" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H9" s="30" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K9" s="24" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="L9" s="25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>OVHcloud, T-Systems, STACKIT, Scaleway, S3NS (Thales-Google JV); ~80% of EU sovereign cloud</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>AWS Sovereign Cloud (GA Jan 2026), Azure sovereign controls; ~20% via US sovereign offerings</t>
+        </is>
+      </c>
+      <c r="O9" s="31" t="inlineStr">
+        <is>
+          <t>Broadcom sovereign cloud report; EC €180M tender Apr 2026; EU sovereign cloud projected to reach €100bn by 2031</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>AI DATACENTERS</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Data Center Market (Total: colocation, hyperscale, enterprise)</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="n">
+        <v>270</v>
+      </c>
+      <c r="D10" s="32" t="n">
+        <v>301</v>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>69</v>
+      </c>
+      <c r="F10" s="32" t="n">
+        <v>77</v>
+      </c>
+      <c r="G10" s="33" t="n">
+        <v>0.2555555555555555</v>
+      </c>
+      <c r="H10" s="33" t="n">
+        <v>0.2558139534883721</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="J10" s="23" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="K10" s="24" t="n">
+        <v>0.2507246376811594</v>
+      </c>
+      <c r="L10" s="25" t="n">
+        <v>0.7507246376811594</v>
+      </c>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>Equinix (US-HQ, ~$5bn EU rev), Digital Realty (US-HQ, ~$2bn EU rev), EU telecoms, Interxion; ~25% EU-HQ</t>
+        </is>
+      </c>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>AWS, Microsoft, Google build ~60% of new EU capacity; US-HQ operators dominate hyperscale segment</t>
+        </is>
+      </c>
+      <c r="O10" s="34" t="inlineStr">
+        <is>
+          <t>Fortune BI; Mordor Intel; EU at ~25.6% of global; hyperscale self-built fastest growing at 19% CAGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>AI DATACENTERS</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Data Center Colocation (EU only)</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F11" s="32" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="G11" s="36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" s="36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="23" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="K11" s="24" t="n">
+        <v>0.2489626556016597</v>
+      </c>
+      <c r="L11" s="25" t="n">
+        <v>0.7510373443983402</v>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>Interxion/Digital Realty (US-HQ), DATA4, AtosOrigin, EU telecoms; ~25% EU-HQ operators</t>
+        </is>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>Equinix (US), Digital Realty (US), CyrusOne (US), NTT (Japan) dominate EU colocation; ~75% non-EU HQ</t>
+        </is>
+      </c>
+      <c r="O11" s="34" t="inlineStr">
+        <is>
+          <t>Research &amp; Markets Q2 2026; growing 17.3% YoY; AI/GPU workloads key driver</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>AI DATACENTERS</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>AI Accelerator / GPU Market</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="n">
+        <v>160</v>
+      </c>
+      <c r="D12" s="32" t="n">
+        <v>200</v>
+      </c>
+      <c r="E12" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="F12" s="32" t="n">
+        <v>22</v>
+      </c>
+      <c r="G12" s="33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H12" s="33" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="I12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="K12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>No EU AI accelerator at scale; Axelera AI (&lt;$50M), SiPearl (&lt;$20M) are early-stage</t>
+        </is>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>NVIDIA (~80% share = ~$12.8bn EU), AMD (~7%), Google TPU, AWS Trainium, Broadcom ASICs</t>
+        </is>
+      </c>
+      <c r="O12" s="34" t="inlineStr">
+        <is>
+          <t>Silicon Analysts; EU ~10% of global AI accelerator consumption; 100% imported; US export control risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>LLMs</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>LLM Market (Models, APIs, Enterprise SW)</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="37" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="37" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G13" s="38" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H13" s="38" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J13" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K13" s="24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L13" s="25" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>Mistral AI ($400M ARR, ~60% from EU = ~$240M EU); Aleph Alpha (~$30M EU); others ~$230M</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>OpenAI (~29% share), Anthropic (~31% share), Google, Meta, xAI; ~75% of EU LLM spend goes to US providers</t>
+        </is>
+      </c>
+      <c r="O13" s="39" t="inlineStr">
+        <is>
+          <t>AllTechMagazine; Precedence Research; Mistral targeting $1bn rev 2026; EU ~20% of global LLM market</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>LLMs</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>AI Infrastructure Spend (Training + Inference Compute)</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="n">
+        <v>581.7</v>
+      </c>
+      <c r="D14" s="37" t="n">
+        <v>700</v>
+      </c>
+      <c r="E14" s="37" t="n">
+        <v>58</v>
+      </c>
+      <c r="F14" s="37" t="n">
+        <v>70</v>
+      </c>
+      <c r="G14" s="38" t="n">
+        <v>0.09970775313735601</v>
+      </c>
+      <c r="H14" s="38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I14" s="22" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="J14" s="23" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="K14" s="24" t="n">
+        <v>0.09999999999999999</v>
+      </c>
+      <c r="L14" s="25" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>EuroHPC (€7bn budget), Mistral Compute JV, EU national AI compute; ~10% of EU AI infra spend is EU-controlled</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>NVIDIA, US hyperscalers (AWS/Azure/GCP), AMD provide ~90% of EU AI compute infrastructure</t>
+        </is>
+      </c>
+      <c r="O14" s="39" t="inlineStr">
+        <is>
+          <t>Gartner 2026; AllTechMagazine; EU ~10% of global; mostly consumed via US cloud platforms</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>QUANTUM</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Quantum Computing (Hardware, Software, Services)</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D15" s="40" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E15" s="40" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F15" s="40" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G15" s="41" t="n">
+        <v>0.2526315789473684</v>
+      </c>
+      <c r="H15" s="41" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="I15" s="22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J15" s="23" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K15" s="24" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="L15" s="25" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="M15" s="12" t="inlineStr">
+        <is>
+          <t>IQM ($36M / ~€31M global), Pasqal (€16.5M commercial), AQT, QuiX (~$10M combined); ~42% EU-HQ share of EU market</t>
+        </is>
+      </c>
+      <c r="N15" s="12" t="inlineStr">
+        <is>
+          <t>IBM Quantum, Google, Amazon Braket, IonQ ($130M global), Quantinuum, D-Wave; ~58% of EU quantum spend</t>
+        </is>
+      </c>
+      <c r="O15" s="42" t="inlineStr">
+        <is>
+          <t>QED-C 2026 Report; Precedence Research; Europe ~25% of global quantum market; EU companies competitive</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>QUANTUM</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Quantum Sensing &amp; Communications</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D16" s="40" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E16" s="40" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F16" s="40" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G16" s="41" t="n">
+        <v>0.297872340425532</v>
+      </c>
+      <c r="H16" s="41" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I16" s="22" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J16" s="23" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K16" s="24" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="L16" s="25" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="M16" s="12" t="inlineStr">
+        <is>
+          <t>ID Quantique (Swiss), Thales, Airbus Defence, EU quantum startups; ~57% EU-HQ share</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>US defence contractors, Toshiba (Japan) in QKD; ~43% non-EU</t>
+        </is>
+      </c>
+      <c r="O16" s="42" t="inlineStr">
+        <is>
+          <t>QED-C 2026 Report; EU strong in quantum sensing/comms, esp. QKD; grows to $1.1bn globally by 2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>QUANTUM</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Cryogenic &amp; Quantum Enabling Equipment</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D17" s="40" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E17" s="40" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F17" s="40" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G17" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H17" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I17" s="22" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J17" s="23" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K17" s="24" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L17" s="25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M17" s="12" t="inlineStr">
+        <is>
+          <t>Bluefors (Finland, global leader in dilution refrigerators ~$100M+), EU cryo/control electronics startups; ~80% EU-HQ</t>
+        </is>
+      </c>
+      <c r="N17" s="12" t="inlineStr">
+        <is>
+          <t>US enabling tech companies; ~20% non-EU</t>
+        </is>
+      </c>
+      <c r="O17" s="42" t="inlineStr">
+        <is>
+          <t>Industry estimates; Bluefors is dominant global cryogenics supplier; EU strength area</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="inlineStr"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>KEY TAKEAWAYS: EU REVENUE CAPTURE ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>Semiconductor Equipment</t>
+        </is>
+      </c>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t>EU STRENGTH</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ companies (led by ASML) capture ~95% of EU equipment revenue (~$36bn of $38bn). ASML's EUV monopoly is the EU's strongest strategic asset in the entire tech stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1">
+      <c r="A21" s="45" t="inlineStr">
+        <is>
+          <t>Power / Auto / Industrial Chips</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t>EU STRENGTH</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ companies (Infineon, NXP, STMicro) capture ~60% of EU segment revenue (~$16.8bn of $28bn). Strong competitive position in mainstream and specialty chips.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1">
+      <c r="A22" s="45" t="inlineStr">
+        <is>
+          <t>Quantum Enabling Equipment</t>
+        </is>
+      </c>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t>EU STRENGTH</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ companies (Bluefors, startups) capture ~80% of EU segment (~$0.12bn of $0.15bn). Bluefors is the global leader in dilution refrigerators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>Sovereign Cloud</t>
+        </is>
+      </c>
+      <c r="B23" s="47" t="inlineStr">
+        <is>
+          <t>EU MODERATE</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ providers capture ~80% of emerging sovereign cloud segment (~$2.8bn of $3.5bn). Growing fast from small base; EC tender sets precedent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="48" t="inlineStr">
+        <is>
+          <t>Quantum Computing</t>
+        </is>
+      </c>
+      <c r="B24" s="47" t="inlineStr">
+        <is>
+          <t>EU MODERATE</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ companies (IQM, Pasqal, AQT, QuiX) capture ~42% of EU quantum market (~$0.20bn of $0.48bn). Competitive but US platforms dominate cloud access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>Cloud Infrastructure (IaaS/PaaS)</t>
+        </is>
+      </c>
+      <c r="B25" s="50" t="inlineStr">
+        <is>
+          <t>EU WEAK</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ providers capture only ~15% of EU cloud infra market (~$13.1bn of $87bn). US hyperscalers invest €10bn/quarter in EU, making gap structurally unbridgeable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>LLMs / AI Models</t>
+        </is>
+      </c>
+      <c r="B26" s="50" t="inlineStr">
+        <is>
+          <t>EU WEAK</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>EU companies (led by Mistral) capture ~25% of EU LLM spend (~$0.5bn of $2bn). Mistral growing fast but US models (OpenAI, Anthropic, Google) dominate enterprise use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="35" customHeight="1">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>AI Accelerators / GPUs</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="inlineStr">
+        <is>
+          <t>EU CRITICAL GAP</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ companies capture 0% of EU AI accelerator spend (~$0 of $16bn). Total dependency on NVIDIA/AMD. No EU company produces AI GPUs at scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>AI Chips (Logic + Memory)</t>
+        </is>
+      </c>
+      <c r="B28" s="51" t="inlineStr">
+        <is>
+          <t>EU CRITICAL GAP</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ companies capture 0% of EU AI chip consumption (~$0 of $5bn). EU has no leading-edge AI chip design or HBM memory production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="35" customHeight="1">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>AI Infrastructure</t>
+        </is>
+      </c>
+      <c r="B29" s="51" t="inlineStr">
+        <is>
+          <t>EU CRITICAL GAP</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>EU-controlled compute is only ~10% of EU AI infrastructure spend (~$5.8bn of $58bn). 90% flows through US cloud platforms and US-designed hardware.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O17"/>
+  <mergeCells count="12">
+    <mergeCell ref="C28:O28"/>
+    <mergeCell ref="C27:O27"/>
+    <mergeCell ref="C22:O22"/>
+    <mergeCell ref="C23:O23"/>
+    <mergeCell ref="A19:O19"/>
+    <mergeCell ref="C20:O20"/>
+    <mergeCell ref="C26:O26"/>
+    <mergeCell ref="C29:O29"/>
+    <mergeCell ref="C21:O21"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="C25:O25"/>
+    <mergeCell ref="C24:O24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Market Sizing tab: 2035 forecasts + growth & self-reliance columns
Major update to Sheet 3 (Market Sizing & EU Revenue):
- Replaced 2026E estimates with 2035E forecasts across all 16 segments
- Added 'Base Case Growth Expectations Through 2035' column (light blue)
  with CAGR projections, market structure shifts, and demand drivers
- Added 'What EU Needs to Do for Self-Reliance by 2035' column (purple)
  with specific policy actions, investment targets, and measurable goals

2035 market projections sourced from Precedence Research, SNS Insider,
Research & Markets, Kaiso Research, Vantage Market Research, QED-C,
Future Market Insights, Expert Market Research, and others.

Row heights increased to 120px to accommodate the narrative columns.
Summary takeaways updated with 2035 self-reliance roadmap targets.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EU_Chips_Act_2.0_Dependency_Analysis.xlsx
+++ b/EU_Chips_Act_2.0_Dependency_Analysis.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dependency Analysis'!$A$1:$N$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Market Sizing &amp; EU Revenue'!$A$1:$O$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Market Sizing &amp; EU Revenue'!$A$1:$Q$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -85,7 +85,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -172,6 +172,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DAEEF3"/>
+        <bgColor rgb="00DAEEF3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6E0EC"/>
+        <bgColor rgb="00E6E0EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
         <bgColor rgb="001F3864"/>
       </patternFill>
@@ -209,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -286,14 +298,14 @@
     <xf numFmtId="165" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
@@ -337,20 +349,20 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3421,7 +3433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3438,7 +3450,9 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="45" customWidth="1" min="13" max="13"/>
     <col width="45" customWidth="1" min="14" max="14"/>
-    <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="55" customWidth="1" min="15" max="15"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
+    <col width="50" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="55" customHeight="1">
@@ -3454,83 +3468,81 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>GLOBAL MARKET SIZE 2025
-(USD bn)</t>
+          <t>GLOBAL MARKET SIZE 2025 (USD bn)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>GLOBAL MARKET SIZE 2026E
-(USD bn)</t>
+          <t>GLOBAL MARKET SIZE 2035E (USD bn)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>EU MARKET SIZE 2025
-(USD bn)</t>
+          <t>EU MARKET SIZE 2025 (USD bn)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>EU MARKET SIZE 2026E
-(USD bn)</t>
+          <t>EU MARKET SIZE 2035E (USD bn)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>EU AS % OF
-GLOBAL (2025)</t>
+          <t>EU AS % OF GLOBAL (2025)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>EU AS % OF
-GLOBAL (2026E)</t>
+          <t>EU AS % OF GLOBAL (2035E)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>EU REVENUE CAPTURED BY
-EU-HQ COMPANIES (USD bn, 2025)</t>
+          <t>EU REVENUE CAPTURED BY EU-HQ COMPANIES (USD bn 2025)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>EU REVENUE CAPTURED BY
-NON-EU COMPANIES (USD bn, 2025)</t>
+          <t>EU REVENUE CAPTURED BY NON-EU COMPANIES (USD bn 2025)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>% CAPTURED BY
-EU COMPANIES</t>
+          <t>% CAPTURED BY EU COMPANIES</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>% CAPTURED BY
-NON-EU COMPANIES</t>
+          <t>% CAPTURED BY NON-EU COMPANIES</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>KEY EU COMPANIES
-(Revenue, 2025)</t>
+          <t>KEY EU COMPANIES (Revenue 2025)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>KEY NON-EU COMPANIES
-(Share of EU Market)</t>
+          <t>KEY NON-EU COMPANIES (Share of EU Market)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>BASE CASE GROWTH EXPECTATIONS THROUGH 2035</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>WHAT EU NEEDS TO DO FOR SELF-RELIANCE BY 2035</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>SOURCE / NOTES</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="70" customHeight="1">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>SEMICONDUCTORS</t>
@@ -3545,19 +3557,19 @@
         <v>791.7</v>
       </c>
       <c r="D2" s="20" t="n">
-        <v>975</v>
+        <v>1280</v>
       </c>
       <c r="E2" s="20" t="n">
         <v>54.5</v>
       </c>
       <c r="F2" s="20" t="n">
-        <v>60.4</v>
+        <v>130</v>
       </c>
       <c r="G2" s="21" t="n">
-        <v>0.06883920677024125</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H2" s="21" t="n">
-        <v>0.06194871794871794</v>
+        <v>0.102</v>
       </c>
       <c r="I2" s="22" t="n">
         <v>16</v>
@@ -3566,14 +3578,14 @@
         <v>38.5</v>
       </c>
       <c r="K2" s="24" t="n">
-        <v>0.2935779816513762</v>
+        <v>0.29</v>
       </c>
       <c r="L2" s="25" t="n">
-        <v>0.7064220183486238</v>
+        <v>0.71</v>
       </c>
       <c r="M2" s="15" t="inlineStr">
         <is>
-          <t>Infineon (€14.7bn global), NXP ($12.3bn global), STMicro ($11.8bn global); combined EU-market share ~30%</t>
+          <t>Infineon (EUR14.7bn global), NXP ($12.3bn global), STMicro ($11.8bn global); combined EU-market share ~30%</t>
         </is>
       </c>
       <c r="N2" s="15" t="inlineStr">
@@ -3583,11 +3595,21 @@
       </c>
       <c r="O2" s="26" t="inlineStr">
         <is>
-          <t>SIA/WSTS 2025 actuals; WSTS Autumn 2026 forecast ($975bn); ESIA Europe data ($54.5bn)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="70" customHeight="1">
+          <t>Global market grows at ~5-7% CAGR to $1.1-1.4T by 2035. AI logic and memory drive &gt;60% of revenue growth. EU share of global production rises from ~10% to 15-20% if Chips Act 2.0 targets are met. Automotive and power electronics remain EU strength segments, growing at 8-9% CAGR.</t>
+        </is>
+      </c>
+      <c r="P2" s="27" t="inlineStr">
+        <is>
+          <t>EU must operationalise the 3nm open foundry by 2033 and ramp to volume by 2035. Must reach 20% global production share (Chips Act target). Requires EUR 120bn mobilisation on schedule, coordinated demand from AI Gigafactories and CADA. Must build integrated design-to-packaging capability rather than isolated fab capacity. Workforce gap of 30-50K must be closed through competence centres and immigration reform.</t>
+        </is>
+      </c>
+      <c r="Q2" s="28" t="inlineStr">
+        <is>
+          <t>SIA/WSTS 2025 actuals; Precedence Research 2035 forecast ($1,277bn); Expert Market Research ($1,413bn); EU share assumes Chips Act 2.0 targets partially met</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
           <t>SEMICONDUCTORS</t>
@@ -3602,19 +3624,19 @@
         <v>200</v>
       </c>
       <c r="D3" s="20" t="n">
-        <v>280</v>
+        <v>750</v>
       </c>
       <c r="E3" s="20" t="n">
         <v>5</v>
       </c>
       <c r="F3" s="20" t="n">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="G3" s="21" t="n">
         <v>0.025</v>
       </c>
       <c r="H3" s="21" t="n">
-        <v>0.02857142857142857</v>
+        <v>0.1</v>
       </c>
       <c r="I3" s="22" t="n">
         <v>0</v>
@@ -3630,7 +3652,7 @@
       </c>
       <c r="M3" s="15" t="inlineStr">
         <is>
-          <t>No scaled EU AI chip company; Axelera AI, SiPearl are pre-scale (&lt;$50M combined)</t>
+          <t>No scaled EU AI chip company; Axelera AI and SiPearl are pre-scale (&lt;$50M combined)</t>
         </is>
       </c>
       <c r="N3" s="15" t="inlineStr">
@@ -3640,11 +3662,21 @@
       </c>
       <c r="O3" s="26" t="inlineStr">
         <is>
-          <t>Silicon Analysts; Deloitte 2026 Outlook; AI chips ~50% of total semi revenue by value</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="70" customHeight="1">
+          <t>AI chips grow at 14-18% CAGR to $600-1,000bn by 2035, becoming ~55-60% of total semiconductor market. Inference chips overtake training chips by revenue (~65% of AI chip spend by 2035). Custom ASICs grow fastest as hyperscalers verticalise. EU consumption grows 10x as AI Gigafactories and data centres scale up.</t>
+        </is>
+      </c>
+      <c r="P3" s="27" t="inlineStr">
+        <is>
+          <t>EU must develop at least 2-3 scaled AI chip design companies (current startups Axelera, SiPearl must reach &gt;$1bn revenue each). Requires Grand Challenges funding, preferential public procurement, and guaranteed manufacturing access at EU foundry. Must build EU-based EDA toolchain or secure long-term strategic partnership with EDA vendors. Target: 15-20% of EU AI chip consumption sourced from EU-designed chips by 2035.</t>
+        </is>
+      </c>
+      <c r="Q3" s="28" t="inlineStr">
+        <is>
+          <t>Research &amp; Markets ($1T AI accelerator chips by 2035); SNS Insider ($746bn); Deloitte 2026 Outlook; inference shift per Silicon Analysts</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
           <t>SEMICONDUCTORS</t>
@@ -3659,49 +3691,59 @@
         <v>110</v>
       </c>
       <c r="D4" s="20" t="n">
-        <v>125</v>
+        <v>220</v>
       </c>
       <c r="E4" s="20" t="n">
         <v>38</v>
       </c>
       <c r="F4" s="20" t="n">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="G4" s="21" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="H4" s="21" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="I4" s="22" t="n">
         <v>36</v>
       </c>
-      <c r="H4" s="21" t="n">
+      <c r="J4" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="I4" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J4" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K4" s="24" t="inlineStr">
-        <is>
-          <t>ASML (€32.7bn / ~$35.5bn global rev); Zeiss, BESI, ASM Intl (~$2.5bn combined EU rev)</t>
-        </is>
-      </c>
-      <c r="L4" s="25" t="inlineStr">
+      <c r="K4" s="24" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L4" s="25" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>ASML (EUR32.7bn / ~$35.5bn global rev); Zeiss, BESI, ASM Intl (~$2.5bn combined EU rev)</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="inlineStr">
         <is>
           <t>Applied Materials, Lam Research, Tokyo Electron, KLA, Screen (~$2bn EU-origin rev)</t>
         </is>
       </c>
-      <c r="M4" s="15" t="inlineStr">
-        <is>
-          <t>ASML Annual Report 2025; EU dominates via ASML EUV monopoly; equipment is EU strength area</t>
-        </is>
-      </c>
-      <c r="N4" s="15" t="inlineStr"/>
-      <c r="O4" s="26" t="inlineStr"/>
-    </row>
-    <row r="5" ht="70" customHeight="1">
+      <c r="O4" s="26" t="inlineStr">
+        <is>
+          <t>Equipment market grows at ~7% CAGR to ~$220bn by 2035. EUV and High-NA EUV demand accelerates as sub-3nm nodes proliferate. ASML revenue target $44-60bn by 2030. Advanced packaging equipment segment grows fastest at 12-15% CAGR. EU maintains dominant position through ASML monopoly.</t>
+        </is>
+      </c>
+      <c r="P4" s="27" t="inlineStr">
+        <is>
+          <t>EU must maintain and extend ASML's technological lead (High-NA EUV and beyond). Must develop EU-based capabilities in etch, deposition, and inspection to reduce dependence on Applied Materials/Lam Research/TEL. Should invest in advanced packaging equipment (currently Asia-dominated). Must manage export control alignment with allies carefully to preserve commercial viability while protecting security interests.</t>
+        </is>
+      </c>
+      <c r="Q4" s="28" t="inlineStr">
+        <is>
+          <t>ASML Annual Report 2025 (2030 target $44-60bn); industry growth estimates; EU maintains ~35% global equipment revenue share</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
           <t>SEMICONDUCTORS</t>
@@ -3716,49 +3758,59 @@
         <v>95</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>102</v>
+        <v>200</v>
       </c>
       <c r="E5" s="20" t="n">
         <v>28</v>
       </c>
       <c r="F5" s="20" t="n">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="G5" s="21" t="n">
+        <v>0.295</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="I5" s="22" t="n">
         <v>16.8</v>
       </c>
-      <c r="H5" s="21" t="n">
+      <c r="J5" s="23" t="n">
         <v>11.2</v>
       </c>
-      <c r="I5" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J5" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K5" s="24" t="inlineStr">
+      <c r="K5" s="24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L5" s="25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
         <is>
           <t>Infineon (~$10bn EU auto/industrial), NXP (~$5bn EU), STMicro (~$4bn EU); ~60% of EU segment</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="N5" s="15" t="inlineStr">
         <is>
           <t>Texas Instruments, ON Semi, Renesas, Microchip; ~40% of EU power/auto segment</t>
         </is>
       </c>
-      <c r="M5" s="15" t="inlineStr">
-        <is>
-          <t>Company annual reports; EU has strong position in automotive/power semis</t>
-        </is>
-      </c>
-      <c r="N5" s="15" t="inlineStr"/>
-      <c r="O5" s="26" t="inlineStr"/>
-    </row>
-    <row r="6" ht="70" customHeight="1">
+      <c r="O5" s="26" t="inlineStr">
+        <is>
+          <t>Segment grows at ~7-9% CAGR to ~$200bn by 2035, driven by EV penetration reaching 60-70% of new EU car sales, industrial automation, and energy transition (smart grids, renewables). SiC and GaN wide-bandgap semiconductors grow at 20%+ CAGR. EU strengthens position as global automotive chip leader.</t>
+        </is>
+      </c>
+      <c r="P5" s="27" t="inlineStr">
+        <is>
+          <t>EU must defend and extend leadership in automotive/power chips. Requires continued investment in SiC/GaN fab capacity (Infineon, STMicro expanding). Must capture AI-in-vehicle chip opportunity (edge inference for autonomous driving). Should leverage automotive OEM relationships to create demand pull for EU-designed chips. Ensure raw material supply (SiC substrates, gallium) via Critical Raw Materials Act diversification.</t>
+        </is>
+      </c>
+      <c r="Q5" s="28" t="inlineStr">
+        <is>
+          <t>Company annual reports; EU automotive chip share grows as EV adoption accelerates; SiC/GaN CAGR from industry consensus</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
           <t>SEMICONDUCTORS</t>
@@ -3773,19 +3825,19 @@
         <v>28</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>45</v>
+        <v>150</v>
       </c>
       <c r="E6" s="20" t="n">
         <v>1.5</v>
       </c>
       <c r="F6" s="20" t="n">
-        <v>2.5</v>
+        <v>15</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.05400000000000001</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>0.05555555555555555</v>
+        <v>0.1</v>
       </c>
       <c r="I6" s="22" t="n">
         <v>0</v>
@@ -3811,11 +3863,21 @@
       </c>
       <c r="O6" s="26" t="inlineStr">
         <is>
-          <t>Deloitte; industry estimates; HBM critical for AI training/inference</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="70" customHeight="1">
+          <t>HBM market grows at ~18-20% CAGR to $120-180bn by 2035 as AI training/inference scales. HBM4 and HBM5 generations increase bandwidth and capacity. Memory becomes bottleneck for AI compute scaling. EU consumption grows 10x with AI Gigafactory buildout but remains 100% import-dependent without intervention.</t>
+        </is>
+      </c>
+      <c r="P6" s="27" t="inlineStr">
+        <is>
+          <t>EU must establish domestic memory R&amp;D and pilot production capability. Could pursue strategic partnership with one major memory manufacturer (SK Hynix, Samsung, or Micron) for EU-based HBM packaging facility. Should fund advanced memory research through Chips for Europe Initiative. Minimum viable goal: EU-based HBM packaging/testing by 2032, capturing 10-15% of EU HBM consumption. Full domestic production is unrealistic by 2035.</t>
+        </is>
+      </c>
+      <c r="Q6" s="28" t="inlineStr">
+        <is>
+          <t>Deloitte; industry estimates; HBM CAGR from memory market analysis; EU consumption scales with AI Gigafactories</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>CLOUD</t>
@@ -3830,19 +3892,19 @@
         <v>350</v>
       </c>
       <c r="D7" s="29" t="n">
-        <v>435</v>
+        <v>1200</v>
       </c>
       <c r="E7" s="29" t="n">
         <v>87</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>108</v>
+        <v>300</v>
       </c>
       <c r="G7" s="30" t="n">
-        <v>0.2485714285714286</v>
+        <v>0.249</v>
       </c>
       <c r="H7" s="30" t="n">
-        <v>0.2482758620689655</v>
+        <v>0.25</v>
       </c>
       <c r="I7" s="22" t="n">
         <v>13.1</v>
@@ -3851,10 +3913,10 @@
         <v>73.90000000000001</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>0.1505747126436782</v>
+        <v>0.15</v>
       </c>
       <c r="L7" s="25" t="n">
-        <v>0.8494252873563219</v>
+        <v>0.85</v>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
@@ -3866,13 +3928,23 @@
           <t>AWS (~30%), Azure (~25%), Google Cloud (~15%); combined ~70% of EU cloud infra = ~$61bn</t>
         </is>
       </c>
-      <c r="O7" s="31" t="inlineStr">
-        <is>
-          <t>Synergy Research Group 2025; EU market ~€61bn ($70bn) in 2024, growing 24% YoY; EU providers at 15% share</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="70" customHeight="1">
+      <c r="O7" s="26" t="inlineStr">
+        <is>
+          <t>Cloud infra grows at ~13-15% CAGR to $1,000-1,400bn by 2035. AI workloads drive majority of incremental growth. EU market grows ~3.4x from $87bn to ~$300bn. EU provider market share unlikely to exceed 20% without massive intervention; US hyperscalers continue investing EUR 10bn/quarter in EU. Sovereign cloud segment grows fastest at 25-30% CAGR.</t>
+        </is>
+      </c>
+      <c r="P7" s="27" t="inlineStr">
+        <is>
+          <t>EU must implement CADA sovereignty framework (SEAL levels) and enforce mandatory risk assessments for public-sector cloud procurement. Must triple data centre capacity as planned. Should create interoperable EU cloud standards (GAIA-X evolution). Target: EU providers capture 25-30% of EU cloud market by 2035 (up from 15%). Sovereign cloud must reach EUR 100bn+ and become default for public sector. Open-source-first principle critical for reducing vendor lock-in.</t>
+        </is>
+      </c>
+      <c r="Q7" s="31" t="inlineStr">
+        <is>
+          <t>Future Market Insights ($2,649bn global by 2035); Expert Market Research ($2,478bn); Synergy Research EU share data; CADA tripling target</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>CLOUD</t>
@@ -3887,13 +3959,13 @@
         <v>430</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>500</v>
+        <v>1800</v>
       </c>
       <c r="E8" s="29" t="n">
         <v>86</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>100</v>
+        <v>360</v>
       </c>
       <c r="G8" s="30" t="n">
         <v>0.2</v>
@@ -3908,7 +3980,7 @@
         <v>77.40000000000001</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1</v>
       </c>
       <c r="L8" s="25" t="n">
         <v>0.9</v>
@@ -3923,13 +3995,23 @@
           <t>Microsoft 365, Salesforce, Google Workspace, ServiceNow, Oracle; ~90% of EU SaaS spend</t>
         </is>
       </c>
-      <c r="O8" s="31" t="inlineStr">
-        <is>
-          <t>Grand View Research; Fortune BI; SAP is largest EU SaaS provider; US dominance even more acute than IaaS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="70" customHeight="1">
+      <c r="O8" s="26" t="inlineStr">
+        <is>
+          <t>SaaS grows at ~15-16% CAGR to $1,500-2,000bn by 2035. AI-native SaaS (embedded LLMs, copilots) becomes dominant delivery model. EU market grows ~4x to ~$360bn. EU provider share remains under pressure at ~10% without structural change. Enterprise switching costs and ecosystem lock-in favour incumbents.</t>
+        </is>
+      </c>
+      <c r="P8" s="27" t="inlineStr">
+        <is>
+          <t>EU must invest in open-source AI-powered SaaS alternatives for critical government and enterprise functions. Should leverage EU Open Source Strategy and open-source-first procurement principle. SAP must maintain/grow EU market leadership in ERP. EU should nurture next-generation AI-native SaaS startups through public procurement and Chips Fund-type venture support. Target: 15-20% EU provider share by 2035. Self-reliance in SaaS is the hardest segment to achieve.</t>
+        </is>
+      </c>
+      <c r="Q8" s="31" t="inlineStr">
+        <is>
+          <t>ResearchAndMarkets ($3.5T total cloud by 2035); SaaS ~50% of total cloud; EU share remains structurally challenged</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="120" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>CLOUD</t>
@@ -3944,13 +4026,13 @@
         <v>5</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="E9" s="29" t="n">
         <v>3.5</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>5.6</v>
+        <v>70</v>
       </c>
       <c r="G9" s="30" t="n">
         <v>0.7</v>
@@ -3965,7 +4047,7 @@
         <v>0.7</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="L9" s="25" t="n">
         <v>0.2</v>
@@ -3980,13 +4062,23 @@
           <t>AWS Sovereign Cloud (GA Jan 2026), Azure sovereign controls; ~20% via US sovereign offerings</t>
         </is>
       </c>
-      <c r="O9" s="31" t="inlineStr">
-        <is>
-          <t>Broadcom sovereign cloud report; EC €180M tender Apr 2026; EU sovereign cloud projected to reach €100bn by 2031</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1">
+      <c r="O9" s="26" t="inlineStr">
+        <is>
+          <t>Sovereign cloud grows at ~35% CAGR from small base to $80-120bn globally by 2035. EU is largest sovereign cloud market (70% of global). EU sovereign cloud projected to reach EUR 100bn by 2031, and continue growing. CIO demand strong: 60% of Western European CIOs want more local cloud providers. SEAL framework drives government adoption.</t>
+        </is>
+      </c>
+      <c r="P9" s="27" t="inlineStr">
+        <is>
+          <t>EU must fully implement CADA SEAL framework and make SEAL-3/SEAL-4 mandatory for sensitive public-sector workloads by 2028. Must ensure 4+ competitive EU sovereign cloud providers scale to EUR 10bn+ revenue each. Should standardise sovereign cloud APIs for portability. Must resolve S3NS-type hybrid arrangements (Thales-Google JV) - determine if these truly count as sovereign. Target: EU-controlled sovereign cloud captures 85%+ of EU public-sector cloud spend by 2035.</t>
+        </is>
+      </c>
+      <c r="Q9" s="31" t="inlineStr">
+        <is>
+          <t>Broadcom sovereign cloud report; Precedence Research sovereign AI infra ($177bn by 2035); EC EUR180M tender precedent</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>AI DATACENTERS</t>
@@ -4001,19 +4093,19 @@
         <v>270</v>
       </c>
       <c r="D10" s="32" t="n">
-        <v>301</v>
+        <v>900</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>69</v>
       </c>
       <c r="F10" s="32" t="n">
-        <v>77</v>
+        <v>230</v>
       </c>
       <c r="G10" s="33" t="n">
-        <v>0.2555555555555555</v>
+        <v>0.256</v>
       </c>
       <c r="H10" s="33" t="n">
-        <v>0.2558139534883721</v>
+        <v>0.256</v>
       </c>
       <c r="I10" s="22" t="n">
         <v>17.3</v>
@@ -4022,10 +4114,10 @@
         <v>51.8</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>0.2507246376811594</v>
+        <v>0.25</v>
       </c>
       <c r="L10" s="25" t="n">
-        <v>0.7507246376811594</v>
+        <v>0.75</v>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
@@ -4037,13 +4129,23 @@
           <t>AWS, Microsoft, Google build ~60% of new EU capacity; US-HQ operators dominate hyperscale segment</t>
         </is>
       </c>
-      <c r="O10" s="34" t="inlineStr">
-        <is>
-          <t>Fortune BI; Mordor Intel; EU at ~25.6% of global; hyperscale self-built fastest growing at 19% CAGR</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="70" customHeight="1">
+      <c r="O10" s="26" t="inlineStr">
+        <is>
+          <t>Global DC market grows at ~11-13% CAGR to $700-1,000bn by 2035. AI-dedicated capacity grows at 25%+ CAGR. EU data centre capacity triples per CADA target (from 3.6 GW to ~11 GW by 2033). Energy becomes binding constraint: grid capacity, renewable supply, and cooling technology are key bottlenecks. Secondary EU markets (Spain, Poland, Nordics) grow fastest.</t>
+        </is>
+      </c>
+      <c r="P10" s="27" t="inlineStr">
+        <is>
+          <t>EU must deliver CADA tripling target and resolve energy bottleneck through Strategic Roadmap for Digitalisation and AI in Energy. Must streamline permitting (12-month max under Chips Act 2.0 model). Should incentivise EU-HQ data centre operators to scale up. Must ensure new capacity uses EU-designed chips when available (linking CADA to Chips Act 2.0 demand side). Target: EU-HQ operators capture 35-40% of EU DC market by 2035 (up from 25%).</t>
+        </is>
+      </c>
+      <c r="Q10" s="34" t="inlineStr">
+        <is>
+          <t>Spherical Insights ($988bn by 2035); SNS Insider ($882bn); Fortune BI; CADA tripling target; EU energy constraint analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>AI DATACENTERS</t>
@@ -4068,7 +4170,7 @@
         <v>24.1</v>
       </c>
       <c r="F11" s="32" t="n">
-        <v>28.3</v>
+        <v>106</v>
       </c>
       <c r="G11" s="36" t="inlineStr">
         <is>
@@ -4087,10 +4189,10 @@
         <v>18.1</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.2489626556016597</v>
+        <v>0.25</v>
       </c>
       <c r="L11" s="25" t="n">
-        <v>0.7510373443983402</v>
+        <v>0.75</v>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
@@ -4102,13 +4204,23 @@
           <t>Equinix (US), Digital Realty (US), CyrusOne (US), NTT (Japan) dominate EU colocation; ~75% non-EU HQ</t>
         </is>
       </c>
-      <c r="O11" s="34" t="inlineStr">
-        <is>
-          <t>Research &amp; Markets Q2 2026; growing 17.3% YoY; AI/GPU workloads key driver</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="70" customHeight="1">
+      <c r="O11" s="26" t="inlineStr">
+        <is>
+          <t>EU colocation grows at ~12-15% CAGR to ~$100-110bn by 2035. AI and GPU workloads become &gt;40% of colocation revenue. Wholesale colocation grows faster than retail as hyperscalers lease rather than build. Power density requirements increase from 10-15 kW/rack to 50-100+ kW/rack for AI. Liquid cooling becomes standard.</t>
+        </is>
+      </c>
+      <c r="P11" s="27" t="inlineStr">
+        <is>
+          <t>EU must develop EU-headquartered colocation champions through public procurement preferences and strategic project designation. Should require EU data sovereignty compliance for colocation hosting government/critical infrastructure workloads. Must invest in liquid cooling and high-density infrastructure R&amp;D. Target: EU-HQ colocation operators capture 35% of EU market by 2035 (up from 25%).</t>
+        </is>
+      </c>
+      <c r="Q11" s="34" t="inlineStr">
+        <is>
+          <t>NextMSC ($106bn EU colocation by 2035); Research &amp; Markets; AI workload shift drives density and revenue growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="120" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>AI DATACENTERS</t>
@@ -4123,19 +4235,19 @@
         <v>160</v>
       </c>
       <c r="D12" s="32" t="n">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="E12" s="32" t="n">
         <v>16</v>
       </c>
       <c r="F12" s="32" t="n">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="G12" s="33" t="n">
         <v>0.1</v>
       </c>
       <c r="H12" s="33" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="I12" s="22" t="n">
         <v>0</v>
@@ -4151,7 +4263,7 @@
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>No EU AI accelerator at scale; Axelera AI (&lt;$50M), SiPearl (&lt;$20M) are early-stage</t>
+          <t>No EU AI accelerator at scale; Axelera AI (&lt;$50M) and SiPearl (&lt;$20M) are early-stage</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
@@ -4159,13 +4271,23 @@
           <t>NVIDIA (~80% share = ~$12.8bn EU), AMD (~7%), Google TPU, AWS Trainium, Broadcom ASICs</t>
         </is>
       </c>
-      <c r="O12" s="34" t="inlineStr">
-        <is>
-          <t>Silicon Analysts; EU ~10% of global AI accelerator consumption; 100% imported; US export control risk</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="70" customHeight="1">
+      <c r="O12" s="26" t="inlineStr">
+        <is>
+          <t>AI accelerator market grows at ~17-25% CAGR to $430-1,000bn by 2035. Inference overtakes training as primary spend driver (~65% by 2035). Custom ASICs grow fastest at 30%+ CAGR. NVIDIA share gradually erodes from ~80% to ~55-65% as competition broadens. EU consumption grows 5-6x with AI Gigafactory and data centre expansion.</t>
+        </is>
+      </c>
+      <c r="P12" s="27" t="inlineStr">
+        <is>
+          <t>EU must bring at least 2 EU-designed AI accelerators to volume production by 2032 (Axelera for inference, SiPearl for HPC, or new entrants). Requires preferential public procurement mandating EU silicon in sovereign AI infrastructure. EU foundry must support AI chip manufacturing. Should create RISC-V based open architecture for inference accelerators to avoid CUDA lock-in. Target: EU-designed accelerators capture 10-15% of EU consumption by 2035. Full self-reliance is not achievable; diversified sourcing is realistic goal.</t>
+        </is>
+      </c>
+      <c r="Q12" s="34" t="inlineStr">
+        <is>
+          <t>Research &amp; Markets ($1T by 2035); Kaiso Research ($432bn); SNS Insider ($746bn); inference shift analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>LLMs</t>
@@ -4180,19 +4302,19 @@
         <v>10</v>
       </c>
       <c r="D13" s="37" t="n">
-        <v>12</v>
+        <v>150</v>
       </c>
       <c r="E13" s="37" t="n">
         <v>2</v>
       </c>
       <c r="F13" s="37" t="n">
-        <v>2.5</v>
+        <v>35</v>
       </c>
       <c r="G13" s="38" t="n">
         <v>0.2</v>
       </c>
       <c r="H13" s="38" t="n">
-        <v>0.2083333333333333</v>
+        <v>0.233</v>
       </c>
       <c r="I13" s="22" t="n">
         <v>0.5</v>
@@ -4216,13 +4338,23 @@
           <t>OpenAI (~29% share), Anthropic (~31% share), Google, Meta, xAI; ~75% of EU LLM spend goes to US providers</t>
         </is>
       </c>
-      <c r="O13" s="39" t="inlineStr">
-        <is>
-          <t>AllTechMagazine; Precedence Research; Mistral targeting $1bn rev 2026; EU ~20% of global LLM market</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="70" customHeight="1">
+      <c r="O13" s="26" t="inlineStr">
+        <is>
+          <t>LLM market grows at ~34% CAGR to $150bn by 2035. Market shifts from general-purpose to domain-specific fine-tuned models. Open-weight models gain share vs. proprietary APIs. Inference costs decline 10x, democratising deployment. EU LLM market grows to ~$35bn as enterprise adoption reaches 80%+ penetration. Mistral targets $5-10bn revenue by 2030.</t>
+        </is>
+      </c>
+      <c r="P13" s="27" t="inlineStr">
+        <is>
+          <t>EU must ensure Mistral and other EU model developers reach frontier capability parity. Requires AI Gigafactory compute access for training next-generation models. Must implement open-source-first principle for public-sector AI procurement (CADA). Should fund multilingual EU-specific model development for all 24 official languages. Must build EU model evaluation and safety framework. Target: EU-developed models serve 35-40% of EU LLM market by 2035 (up from 25%).</t>
+        </is>
+      </c>
+      <c r="Q13" s="39" t="inlineStr">
+        <is>
+          <t>Precedence Research ($150bn by 2035); Roots Analysis ($180bn); Mistral revenue trajectory; enterprise AI adoption curves</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>LLMs</t>
@@ -4237,19 +4369,19 @@
         <v>581.7</v>
       </c>
       <c r="D14" s="37" t="n">
-        <v>700</v>
+        <v>2500</v>
       </c>
       <c r="E14" s="37" t="n">
         <v>58</v>
       </c>
       <c r="F14" s="37" t="n">
-        <v>70</v>
+        <v>300</v>
       </c>
       <c r="G14" s="38" t="n">
-        <v>0.09970775313735601</v>
+        <v>0.1</v>
       </c>
       <c r="H14" s="38" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="I14" s="22" t="n">
         <v>5.8</v>
@@ -4258,14 +4390,14 @@
         <v>52.2</v>
       </c>
       <c r="K14" s="24" t="n">
-        <v>0.09999999999999999</v>
+        <v>0.1</v>
       </c>
       <c r="L14" s="25" t="n">
         <v>0.9</v>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>EuroHPC (€7bn budget), Mistral Compute JV, EU national AI compute; ~10% of EU AI infra spend is EU-controlled</t>
+          <t>EuroHPC (EUR7bn budget), Mistral Compute JV, EU national AI compute; ~10% of EU AI infra spend is EU-controlled</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
@@ -4273,13 +4405,23 @@
           <t>NVIDIA, US hyperscalers (AWS/Azure/GCP), AMD provide ~90% of EU AI compute infrastructure</t>
         </is>
       </c>
-      <c r="O14" s="39" t="inlineStr">
-        <is>
-          <t>Gartner 2026; AllTechMagazine; EU ~10% of global; mostly consumed via US cloud platforms</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="70" customHeight="1">
+      <c r="O14" s="26" t="inlineStr">
+        <is>
+          <t>Global AI infrastructure spending grows at ~16% CAGR to $2,000-3,000bn by 2035. Inference infrastructure overtakes training by 2028-2030. Edge AI inference grows at 25%+ CAGR. EU AI infra spend grows 5x to ~$300bn. Currently 90% flows through US platforms; CADA and Chips Act 2.0 aim to redirect significant portion toward EU-controlled infrastructure.</t>
+        </is>
+      </c>
+      <c r="P14" s="27" t="inlineStr">
+        <is>
+          <t>EU must operationalise AI Gigafactories (75,000+ accelerators each) by 2028-2030 as planned. Must build sovereign AI compute layer using EU-designed chips when available. Requires EuroHPC expansion and new Mistral Compute-type JVs. Must train EU workforce in AI infrastructure operations. Should mandate that public-funded AI research uses EU-hosted compute. Target: 25-30% of EU AI infrastructure spend flows through EU-controlled platforms by 2035 (up from 10%).</t>
+        </is>
+      </c>
+      <c r="Q14" s="39" t="inlineStr">
+        <is>
+          <t>Gartner ($2.52T total AI spending in 2026); projected CAGR through 2035; CADA and AI Gigafactory programme targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>QUANTUM</t>
@@ -4294,19 +4436,19 @@
         <v>1.9</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>2.5</v>
+        <v>20</v>
       </c>
       <c r="E15" s="40" t="n">
         <v>0.48</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.63</v>
+        <v>5</v>
       </c>
       <c r="G15" s="41" t="n">
-        <v>0.2526315789473684</v>
+        <v>0.25</v>
       </c>
       <c r="H15" s="41" t="n">
-        <v>0.252</v>
+        <v>0.25</v>
       </c>
       <c r="I15" s="22" t="n">
         <v>0.2</v>
@@ -4315,14 +4457,14 @@
         <v>0.28</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.42</v>
       </c>
       <c r="L15" s="25" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.58</v>
       </c>
       <c r="M15" s="12" t="inlineStr">
         <is>
-          <t>IQM ($36M / ~€31M global), Pasqal (€16.5M commercial), AQT, QuiX (~$10M combined); ~42% EU-HQ share of EU market</t>
+          <t>IQM ($36M / ~EUR31M global), Pasqal (EUR16.5M commercial), AQT, QuiX (~$10M combined); ~42% EU-HQ share of EU market</t>
         </is>
       </c>
       <c r="N15" s="12" t="inlineStr">
@@ -4330,13 +4472,23 @@
           <t>IBM Quantum, Google, Amazon Braket, IonQ ($130M global), Quantinuum, D-Wave; ~58% of EU quantum spend</t>
         </is>
       </c>
-      <c r="O15" s="42" t="inlineStr">
-        <is>
-          <t>QED-C 2026 Report; Precedence Research; Europe ~25% of global quantum market; EU companies competitive</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="70" customHeight="1">
+      <c r="O15" s="26" t="inlineStr">
+        <is>
+          <t>Quantum computing grows at ~27-35% CAGR to $19-46bn by 2035. Fault-tolerant quantum computing expected to emerge by early 2030s. Quantum-as-a-Service becomes dominant delivery model. Pharma, finance, logistics and materials science are first commercial verticals. EU maintains ~25% of global market with strong hardware diversity.</t>
+        </is>
+      </c>
+      <c r="P15" s="27" t="inlineStr">
+        <is>
+          <t>EU must scale IQM, Pasqal, AQT, and QuiX from pilot-line prototypes to commercial-grade production by 2030. Requires Quantum Act coordination with Chips Act 2.0 (shared foundry infrastructure). Must build EU quantum cloud platform to counter IBM/Amazon/Google/Azure dominance. Should industrialise all 6 quantum pilot lines and select 2-3 for commercial fab. Target: EU-HQ companies capture 50%+ of EU quantum market by 2035 (up from 42%).</t>
+        </is>
+      </c>
+      <c r="Q15" s="42" t="inlineStr">
+        <is>
+          <t>Precedence Research ($19.4bn by 2035); Vantage ($45.6bn); SNS Insider ($18.9bn); QED-C 2026 Report; Europe ~25% share maintained</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>QUANTUM</t>
@@ -4351,16 +4503,16 @@
         <v>0.47</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="E16" s="40" t="n">
         <v>0.14</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>0.18</v>
+        <v>0.9</v>
       </c>
       <c r="G16" s="41" t="n">
-        <v>0.297872340425532</v>
+        <v>0.3</v>
       </c>
       <c r="H16" s="41" t="n">
         <v>0.3</v>
@@ -4372,10 +4524,10 @@
         <v>0.06</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.57</v>
       </c>
       <c r="L16" s="25" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.43</v>
       </c>
       <c r="M16" s="12" t="inlineStr">
         <is>
@@ -4387,13 +4539,23 @@
           <t>US defence contractors, Toshiba (Japan) in QKD; ~43% non-EU</t>
         </is>
       </c>
-      <c r="O16" s="42" t="inlineStr">
-        <is>
-          <t>QED-C 2026 Report; EU strong in quantum sensing/comms, esp. QKD; grows to $1.1bn globally by 2028</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="70" customHeight="1">
+      <c r="O16" s="26" t="inlineStr">
+        <is>
+          <t>Quantum sensing grows at ~20% CAGR to $2-4bn by 2035. QKD networks expand as PQC threat drives adoption. Quantum sensors deployed in healthcare (MRI), defence (submarine detection), and infrastructure monitoring. EU has strong academic and industrial base, especially in QKD and atomic sensors.</t>
+        </is>
+      </c>
+      <c r="P16" s="27" t="inlineStr">
+        <is>
+          <t>EU must commercialise QKD technology for critical infrastructure (telecoms, finance, government). Should build pan-EU quantum-secured communication network by 2035 (EuroQCI initiative). Must support quantum sensor startups in navigating defence procurement. Leverage EU strength in photonics (PIXEurope) for integrated quantum sensing chips. Target: EU-HQ companies capture 65%+ of EU quantum sensing/comms market by 2035 (up from 57%).</t>
+        </is>
+      </c>
+      <c r="Q16" s="42" t="inlineStr">
+        <is>
+          <t>QED-C 2026 Report (sensing grows to $1.1bn by 2028); projected 2035 based on continued 18-20% CAGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>QUANTUM</t>
@@ -4408,13 +4570,13 @@
         <v>0.3</v>
       </c>
       <c r="D17" s="40" t="n">
-        <v>0.38</v>
+        <v>1.5</v>
       </c>
       <c r="E17" s="40" t="n">
         <v>0.15</v>
       </c>
       <c r="F17" s="40" t="n">
-        <v>0.19</v>
+        <v>0.75</v>
       </c>
       <c r="G17" s="41" t="n">
         <v>0.5</v>
@@ -4444,207 +4606,213 @@
           <t>US enabling tech companies; ~20% non-EU</t>
         </is>
       </c>
-      <c r="O17" s="42" t="inlineStr">
-        <is>
-          <t>Industry estimates; Bluefors is dominant global cryogenics supplier; EU strength area</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="43" t="inlineStr"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+      <c r="O17" s="26" t="inlineStr">
+        <is>
+          <t>Cryogenic and enabling equipment grows at ~17% CAGR to $1-2bn by 2035 as quantum computing scales. Dilution refrigerator demand grows with every new quantum system deployment. Control electronics and interconnect markets emerge as quantum processors scale beyond 1000 qubits. EU maintains strong position through Bluefors dominance.</t>
+        </is>
+      </c>
+      <c r="P17" s="27" t="inlineStr">
+        <is>
+          <t>EU must maintain Bluefors leadership and expand into adjacent enabling technologies (cryogenic CMOS, photonic interconnects, modular packaging). Chips JU quantum-enabling calls must fund industrialisation not just R&amp;D. Should create EU supply chain for helium-3 (critical for cryogenics). Must develop EU-based quantum control electronics stack. Target: EU-HQ companies maintain 80%+ of EU enabling equipment market and capture 60%+ of global market.</t>
+        </is>
+      </c>
+      <c r="Q17" s="42" t="inlineStr">
+        <is>
+          <t>Industry estimates; Bluefors dominance; Chips JU EUR 20m quantum-enabling call; market scales with quantum system deployments</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>KEY TAKEAWAYS: EU SELF-RELIANCE ROADMAP TO 2035</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
       <c r="A19" s="44" t="inlineStr">
         <is>
-          <t>KEY TAKEAWAYS: EU REVENUE CAPTURE ANALYSIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="35" customHeight="1">
-      <c r="A20" s="45" t="inlineStr">
-        <is>
           <t>Semiconductor Equipment</t>
         </is>
       </c>
-      <c r="B20" s="46" t="inlineStr">
+      <c r="B19" s="45" t="inlineStr">
         <is>
           <t>EU STRENGTH</t>
         </is>
       </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>EU-HQ companies capture ~95% of EU equipment revenue. ASML's High-NA EUV ensures continued dominance through 2035. Maintain lead and expand into adjacent equipment categories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>Power / Auto / Industrial Chips</t>
+        </is>
+      </c>
+      <c r="B20" s="45" t="inlineStr">
+        <is>
+          <t>EU STRENGTH</t>
+        </is>
+      </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ companies (led by ASML) capture ~95% of EU equipment revenue (~$36bn of $38bn). ASML's EUV monopoly is the EU's strongest strategic asset in the entire tech stack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="35" customHeight="1">
-      <c r="A21" s="45" t="inlineStr">
-        <is>
-          <t>Power / Auto / Industrial Chips</t>
-        </is>
-      </c>
-      <c r="B21" s="46" t="inlineStr">
+          <t>EU-HQ companies capture ~60%. EU automotive chip leadership grows with EV transition. SiC/GaN investment and edge AI for vehicles are key growth vectors to reach 65%+ by 2035.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="44" t="inlineStr">
+        <is>
+          <t>Quantum Enabling Equipment</t>
+        </is>
+      </c>
+      <c r="B21" s="45" t="inlineStr">
         <is>
           <t>EU STRENGTH</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ companies (Infineon, NXP, STMicro) capture ~60% of EU segment revenue (~$16.8bn of $28bn). Strong competitive position in mainstream and specialty chips.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="35" customHeight="1">
-      <c r="A22" s="45" t="inlineStr">
-        <is>
-          <t>Quantum Enabling Equipment</t>
+          <t>EU-HQ companies capture ~80%. Bluefors dominance in cryogenics is a global asset. Must industrialise control electronics and interconnects as quantum scales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>Sovereign Cloud</t>
         </is>
       </c>
       <c r="B22" s="46" t="inlineStr">
         <is>
-          <t>EU STRENGTH</t>
+          <t>EU ON TRACK</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ companies (Bluefors, startups) capture ~80% of EU segment (~$0.12bn of $0.15bn). Bluefors is the global leader in dilution refrigerators.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="35" customHeight="1">
-      <c r="A23" s="45" t="inlineStr">
-        <is>
-          <t>Sovereign Cloud</t>
+          <t>EU-HQ capture ~80% of $3.5bn market. Segment grows to ~$70bn EU by 2035. CADA SEAL framework is critical policy lever. Must mandate SEAL-3/4 for public sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="44" t="inlineStr">
+        <is>
+          <t>Quantum Computing</t>
         </is>
       </c>
       <c r="B23" s="47" t="inlineStr">
         <is>
-          <t>EU MODERATE</t>
+          <t>EU COMPETITIVE</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ providers capture ~80% of emerging sovereign cloud segment (~$2.8bn of $3.5bn). Growing fast from small base; EC tender sets precedent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="35" customHeight="1">
-      <c r="A24" s="48" t="inlineStr">
-        <is>
-          <t>Quantum Computing</t>
-        </is>
-      </c>
-      <c r="B24" s="47" t="inlineStr">
-        <is>
-          <t>EU MODERATE</t>
+          <t>EU-HQ capture ~42% of EU market. Must scale IQM/Pasqal to commercial production and build EU quantum cloud. Target: 50%+ by 2035.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="44" t="inlineStr">
+        <is>
+          <t>Cloud Infrastructure</t>
+        </is>
+      </c>
+      <c r="B24" s="48" t="inlineStr">
+        <is>
+          <t>EU CHALLENGED</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ companies (IQM, Pasqal, AQT, QuiX) capture ~42% of EU quantum market (~$0.20bn of $0.48bn). Competitive but US platforms dominate cloud access.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="35" customHeight="1">
-      <c r="A25" s="49" t="inlineStr">
-        <is>
-          <t>Cloud Infrastructure (IaaS/PaaS)</t>
-        </is>
-      </c>
-      <c r="B25" s="50" t="inlineStr">
-        <is>
-          <t>EU WEAK</t>
+          <t>EU-HQ capture only 15% of $87bn EU market. Hyperscaler investment gap is structurally unbridgeable. Sovereign cloud is the realistic path; target 25-30% by 2035.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="44" t="inlineStr">
+        <is>
+          <t>LLMs / AI Models</t>
+        </is>
+      </c>
+      <c r="B25" s="47" t="inlineStr">
+        <is>
+          <t>EU GROWING</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ providers capture only ~15% of EU cloud infra market (~$13.1bn of $87bn). US hyperscalers invest €10bn/quarter in EU, making gap structurally unbridgeable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="35" customHeight="1">
-      <c r="A26" s="49" t="inlineStr">
-        <is>
-          <t>LLMs / AI Models</t>
-        </is>
-      </c>
-      <c r="B26" s="50" t="inlineStr">
-        <is>
-          <t>EU WEAK</t>
+          <t>EU capture ~25% (led by Mistral). Must reach frontier model parity and leverage open-source-first procurement. Target: 35-40% by 2035.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="44" t="inlineStr">
+        <is>
+          <t>AI Accelerators / GPUs</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>EU CRITICAL GAP</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>EU companies (led by Mistral) capture ~25% of EU LLM spend (~$0.5bn of $2bn). Mistral growing fast but US models (OpenAI, Anthropic, Google) dominate enterprise use.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="35" customHeight="1">
-      <c r="A27" s="49" t="inlineStr">
-        <is>
-          <t>AI Accelerators / GPUs</t>
-        </is>
-      </c>
-      <c r="B27" s="51" t="inlineStr">
+          <t>EU capture 0% of $16bn EU market. Must bring 2+ EU-designed accelerators to volume by 2032. Target: 10-15% by 2035. Full self-reliance impossible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="44" t="inlineStr">
+        <is>
+          <t>AI Chips (Logic + Memory)</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
         <is>
           <t>EU CRITICAL GAP</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ companies capture 0% of EU AI accelerator spend (~$0 of $16bn). Total dependency on NVIDIA/AMD. No EU company produces AI GPUs at scale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="35" customHeight="1">
-      <c r="A28" s="49" t="inlineStr">
-        <is>
-          <t>AI Chips (Logic + Memory)</t>
-        </is>
-      </c>
-      <c r="B28" s="51" t="inlineStr">
+          <t>EU capture 0% of $5bn EU market. Foundry (pilot 2030-33) and Grand Challenges are essential. Target: 15-20% of EU consumption by 2035.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="44" t="inlineStr">
+        <is>
+          <t>AI Infrastructure</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
         <is>
           <t>EU CRITICAL GAP</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>EU-HQ companies capture 0% of EU AI chip consumption (~$0 of $5bn). EU has no leading-edge AI chip design or HBM memory production.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="35" customHeight="1">
-      <c r="A29" s="49" t="inlineStr">
-        <is>
-          <t>AI Infrastructure</t>
-        </is>
-      </c>
-      <c r="B29" s="51" t="inlineStr">
-        <is>
-          <t>EU CRITICAL GAP</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>EU-controlled compute is only ~10% of EU AI infrastructure spend (~$5.8bn of $58bn). 90% flows through US cloud platforms and US-designed hardware.</t>
+          <t>EU-controlled is only 10% of $58bn. AI Gigafactories and sovereign compute layer are the path forward. Target: 25-30% by 2035.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O17"/>
-  <mergeCells count="12">
-    <mergeCell ref="C28:O28"/>
-    <mergeCell ref="C27:O27"/>
-    <mergeCell ref="C22:O22"/>
-    <mergeCell ref="C23:O23"/>
-    <mergeCell ref="A19:O19"/>
-    <mergeCell ref="C20:O20"/>
-    <mergeCell ref="C26:O26"/>
-    <mergeCell ref="C29:O29"/>
-    <mergeCell ref="C21:O21"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="C25:O25"/>
-    <mergeCell ref="C24:O24"/>
+  <autoFilter ref="A1:Q17"/>
+  <mergeCells count="11">
+    <mergeCell ref="C21:Q21"/>
+    <mergeCell ref="C20:Q20"/>
+    <mergeCell ref="A18:Q18"/>
+    <mergeCell ref="C25:Q25"/>
+    <mergeCell ref="C24:Q24"/>
+    <mergeCell ref="C28:Q28"/>
+    <mergeCell ref="C27:Q27"/>
+    <mergeCell ref="C19:Q19"/>
+    <mergeCell ref="C23:Q23"/>
+    <mergeCell ref="C22:Q22"/>
+    <mergeCell ref="C26:Q26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>